<commit_message>
Cliff/bumper connector reverse engineered
</commit_message>
<xml_diff>
--- a/kicad/main/STM32G473VCT6_IOs.xlsx
+++ b/kicad/main/STM32G473VCT6_IOs.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="352">
   <si>
     <t>LPQF100</t>
   </si>
@@ -335,6 +335,9 @@
     <t>TIM20_CH3, I2C2_SMBA, FMC_A2, EVENTOUT</t>
   </si>
   <si>
+    <t>LED-PWR</t>
+  </si>
+  <si>
     <t>PA0</t>
   </si>
   <si>
@@ -344,7 +347,7 @@
     <t>ADC12_IN1 , COMP1_INM, COMP3_INP, RTC_TAMP2,WK UP1</t>
   </si>
   <si>
-    <t>ANTI-FALL-LEFT-UP-ADC</t>
+    <t>RR-Q+</t>
   </si>
   <si>
     <t>PA1</t>
@@ -356,7 +359,7 @@
     <t>ADC12_IN2, COMP1_INP, OPAMP1_VINP, OPAMP3_VINP, OPAMP6_VINM</t>
   </si>
   <si>
-    <t>ANTI-FALL-LEFT-DOWN-ADC</t>
+    <t>RF-Q+</t>
   </si>
   <si>
     <t>PA2</t>
@@ -369,7 +372,7 @@
     <t>ADC1_IN3, COMP2_INM, OPAMP1_VOUT, WKUP4/LSCO</t>
   </si>
   <si>
-    <t>ANTI-FALL-RIGHT-UP-ADC</t>
+    <t>LR-Q+</t>
   </si>
   <si>
     <t>VSS</t>
@@ -391,7 +394,7 @@
 1_VINP, OPAMP5_VINM</t>
   </si>
   <si>
-    <t>ANTI-FALL-RIGHT-DOWN-ADC</t>
+    <t>LF-Q+</t>
   </si>
   <si>
     <t>PA4</t>
@@ -403,43 +406,46 @@
     <t>ADC2_IN17, DAC1_OUT1 , COMP1_INM</t>
   </si>
   <si>
+    <t>BUMP-L-Q+</t>
+  </si>
+  <si>
+    <t>MAIN-BRUSH-F-ADC</t>
+  </si>
+  <si>
+    <t>PA5</t>
+  </si>
+  <si>
+    <t>TIM2_CH1 , TIM2_ETR, SPI1_SCK, UCPD1_FRSTX, EVENTOUT</t>
+  </si>
+  <si>
+    <t>ADC2_IN13, DAC1_OUT2, COMP2_INM, OPAMP2_VINM</t>
+  </si>
+  <si>
+    <t>BUMP-R-Q+</t>
+  </si>
+  <si>
+    <t>PA6</t>
+  </si>
+  <si>
+    <t>TIM16_CH1 , TIM3_CH1 , TIM8_BKIN, SPI1_MISO, TIM1_BKIN, COMP1_OUT, QUADSPI1_BK1_IO3, LPUART1_CTS, EVENTOUT</t>
+  </si>
+  <si>
+    <t>ADC2_IN3, DAC2_OUT1 , OPAMP2_VOUT</t>
+  </si>
+  <si>
     <t>MAIN-BRUSH-CURRENT-ADC</t>
   </si>
   <si>
-    <t>MAIN-BRUSH-F-ADC</t>
-  </si>
-  <si>
-    <t>PA5</t>
-  </si>
-  <si>
-    <t>TIM2_CH1 , TIM2_ETR, SPI1_SCK, UCPD1_FRSTX, EVENTOUT</t>
-  </si>
-  <si>
-    <t>ADC2_IN13, DAC1_OUT2, COMP2_INM, OPAMP2_VINM</t>
+    <t>PA7</t>
+  </si>
+  <si>
+    <t>TIM17_CH1 , TIM3_CH2, TIM8_CH1N, SPI1_MOSI, TIM1_CH1 N, COMP2_OUT, QUADSPI1_BK1_IO2, UCPD1_FRSTX, EVENTOUT</t>
+  </si>
+  <si>
+    <t>ADC2_IN4, COMP2_INP, OPAMP1_VINP, OPAMP2_VINP</t>
   </si>
   <si>
     <t>WATER-PUMP-SENSE-ADC</t>
-  </si>
-  <si>
-    <t>PA6</t>
-  </si>
-  <si>
-    <t>TIM16_CH1 , TIM3_CH1 , TIM8_BKIN, SPI1_MISO, TIM1_BKIN, COMP1_OUT, QUADSPI1_BK1_IO3, LPUART1_CTS, EVENTOUT</t>
-  </si>
-  <si>
-    <t>ADC2_IN3, DAC2_OUT1 , OPAMP2_VOUT</t>
-  </si>
-  <si>
-    <t>LED-PWR</t>
-  </si>
-  <si>
-    <t>PA7</t>
-  </si>
-  <si>
-    <t>TIM17_CH1 , TIM3_CH2, TIM8_CH1N, SPI1_MOSI, TIM1_CH1 N, COMP2_OUT, QUADSPI1_BK1_IO2, UCPD1_FRSTX, EVENTOUT</t>
-  </si>
-  <si>
-    <t>ADC2_IN4, COMP2_INP, OPAMP1_VINP, OPAMP2_VINP</t>
   </si>
   <si>
     <t>WHEEL-M-LEFT-IN2</t>
@@ -1846,14 +1852,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <vertAlign val="superscript"/>
+      <vertAlign val="subscript"/>
       <sz val="6"/>
-      <name val="Arial MT"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <color rgb="FF282828"/>
       <name val="Arial MT"/>
       <charset val="1"/>
     </font>
@@ -1864,13 +1864,19 @@
       <charset val="1"/>
     </font>
     <font>
-      <vertAlign val="subscript"/>
       <sz val="6"/>
       <name val="Arial MT"/>
       <charset val="1"/>
     </font>
     <font>
+      <vertAlign val="superscript"/>
       <sz val="6"/>
+      <name val="Arial MT"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF282828"/>
       <name val="Arial MT"/>
       <charset val="1"/>
     </font>
@@ -3574,13 +3580,16 @@
         <v>79</v>
       </c>
       <c r="G21" s="6"/>
+      <c r="H21" s="22" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="22" ht="46.95" customHeight="1" spans="1:14">
       <c r="A22" s="4">
         <v>20</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C22" s="5" t="s">
         <v>9</v>
@@ -3590,13 +3599,13 @@
       </c>
       <c r="E22" s="6"/>
       <c r="F22" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H22" s="22" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="23" ht="46.95" customHeight="1" spans="1:14">
@@ -3604,7 +3613,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>9</v>
@@ -3614,13 +3623,13 @@
       </c>
       <c r="E23" s="6"/>
       <c r="F23" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H23" s="22" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="24" ht="46.95" customHeight="1" spans="1:14">
@@ -3628,7 +3637,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>9</v>
@@ -3638,13 +3647,13 @@
       </c>
       <c r="E24" s="6"/>
       <c r="F24" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H24" s="22" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="25" ht="46.95" customHeight="1" spans="1:14">
@@ -3652,7 +3661,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="17" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C25" s="17" t="s">
         <v>26</v>
@@ -3662,7 +3671,7 @@
       <c r="F25" s="16"/>
       <c r="G25" s="16"/>
       <c r="H25" s="11" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="26" ht="46.95" customHeight="1" spans="1:14">
@@ -3670,7 +3679,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="17" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C26" s="17" t="s">
         <v>26</v>
@@ -3688,7 +3697,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C27" s="8" t="s">
         <v>9</v>
@@ -3698,13 +3707,13 @@
       </c>
       <c r="E27" s="6"/>
       <c r="F27" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H27" s="22" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="28" ht="46.95" customHeight="1" spans="1:14">
@@ -3712,7 +3721,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C28" s="8" t="s">
         <v>9</v>
@@ -3722,15 +3731,18 @@
       </c>
       <c r="E28" s="6"/>
       <c r="F28" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="H28" s="18" t="s">
         <v>102</v>
       </c>
+      <c r="H28" s="1" t="s">
+        <v>103</v>
+      </c>
       <c r="K28" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="N28" s="1" t="s">
         <v>103</v>
       </c>
     </row>
@@ -3739,7 +3751,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C29" s="15" t="s">
         <v>9</v>
@@ -3749,13 +3761,16 @@
       </c>
       <c r="E29" s="16"/>
       <c r="F29" s="17" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G29" s="17" t="s">
-        <v>106</v>
-      </c>
-      <c r="H29" s="22" t="s">
         <v>107</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="N29" s="1" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="30" ht="46.95" customHeight="1" spans="1:14">
@@ -3763,7 +3778,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C30" s="8" t="s">
         <v>9</v>
@@ -3773,13 +3788,13 @@
       </c>
       <c r="E30" s="6"/>
       <c r="F30" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="H30" s="22" t="s">
         <v>111</v>
+      </c>
+      <c r="H30" s="18" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="31" ht="46.95" customHeight="1" spans="1:14">
@@ -3787,7 +3802,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>9</v>
@@ -3797,13 +3812,16 @@
       </c>
       <c r="E31" s="6"/>
       <c r="F31" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
+      </c>
+      <c r="H31" s="22" t="s">
+        <v>116</v>
       </c>
       <c r="N31" s="22" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="32" ht="46.95" customHeight="1" spans="1:14">
@@ -3811,7 +3829,7 @@
         <v>30</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C32" s="15" t="s">
         <v>9</v>
@@ -3821,13 +3839,13 @@
       </c>
       <c r="E32" s="16"/>
       <c r="F32" s="17" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="G32" s="15" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="H32" s="22" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="33" ht="46.95" customHeight="1" spans="1:19">
@@ -3835,7 +3853,7 @@
         <v>31</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>9</v>
@@ -3845,13 +3863,13 @@
       </c>
       <c r="E33" s="6"/>
       <c r="F33" s="5" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H33" s="22" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="34" ht="46.95" customHeight="1" spans="1:19">
@@ -3859,7 +3877,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C34" s="5" t="s">
         <v>9</v>
@@ -3869,13 +3887,13 @@
       </c>
       <c r="E34" s="6"/>
       <c r="F34" s="5" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H34" s="22" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="35" ht="46.95" customHeight="1" spans="1:19">
@@ -3883,7 +3901,7 @@
         <v>33</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C35" s="5" t="s">
         <v>9</v>
@@ -3893,13 +3911,13 @@
       </c>
       <c r="E35" s="6"/>
       <c r="F35" s="5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H35" s="22" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="36" ht="46.95" customHeight="1" spans="1:19">
@@ -3907,7 +3925,7 @@
         <v>34</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C36" s="5" t="s">
         <v>9</v>
@@ -3917,13 +3935,13 @@
       </c>
       <c r="E36" s="6"/>
       <c r="F36" s="23" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H36" s="24" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="37" ht="46.95" customHeight="1" spans="1:19">
@@ -3931,7 +3949,7 @@
         <v>35</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C37" s="5" t="s">
         <v>26</v>
@@ -3941,7 +3959,7 @@
       <c r="F37" s="6"/>
       <c r="G37" s="6"/>
       <c r="H37" s="11" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="38" ht="46.95" customHeight="1" spans="1:19">
@@ -3949,7 +3967,7 @@
         <v>36</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C38" s="5" t="s">
         <v>26</v>
@@ -3958,7 +3976,7 @@
       <c r="E38" s="6"/>
       <c r="F38" s="6"/>
       <c r="G38" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="H38" s="11" t="s">
         <v>27</v>
@@ -3969,7 +3987,7 @@
         <v>37</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C39" s="5" t="s">
         <v>26</v>
@@ -3987,7 +4005,7 @@
         <v>38</v>
       </c>
       <c r="B40" s="15" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C40" s="15" t="s">
         <v>9</v>
@@ -3997,13 +4015,13 @@
       </c>
       <c r="E40" s="16"/>
       <c r="F40" s="17" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="G40" s="17" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="H40" s="22" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="41" ht="46.95" customHeight="1" spans="1:19">
@@ -4011,7 +4029,7 @@
         <v>39</v>
       </c>
       <c r="B41" s="15" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C41" s="15" t="s">
         <v>9</v>
@@ -4021,13 +4039,13 @@
       </c>
       <c r="E41" s="16"/>
       <c r="F41" s="17" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G41" s="17" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="H41" s="22" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="42" ht="46.95" customHeight="1" spans="1:19">
@@ -4035,7 +4053,7 @@
         <v>40</v>
       </c>
       <c r="B42" s="15" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C42" s="15" t="s">
         <v>9</v>
@@ -4045,13 +4063,13 @@
       </c>
       <c r="E42" s="16"/>
       <c r="F42" s="17" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="G42" s="15" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="H42" s="22" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="43" ht="46.95" customHeight="1" spans="1:19">
@@ -4059,7 +4077,7 @@
         <v>41</v>
       </c>
       <c r="B43" s="17" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C43" s="17" t="s">
         <v>9</v>
@@ -4069,13 +4087,13 @@
       </c>
       <c r="E43" s="16"/>
       <c r="F43" s="15" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="G43" s="15" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="H43" s="11" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="44" ht="46.95" customHeight="1" spans="1:19">
@@ -4083,7 +4101,7 @@
         <v>42</v>
       </c>
       <c r="B44" s="17" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C44" s="17" t="s">
         <v>9</v>
@@ -4093,13 +4111,13 @@
       </c>
       <c r="E44" s="16"/>
       <c r="F44" s="17" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="G44" s="17" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="H44" s="11" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="45" ht="46.95" customHeight="1" spans="1:19">
@@ -4107,7 +4125,7 @@
         <v>43</v>
       </c>
       <c r="B45" s="15" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C45" s="15" t="s">
         <v>9</v>
@@ -4117,13 +4135,13 @@
       </c>
       <c r="E45" s="16"/>
       <c r="F45" s="17" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="G45" s="15" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="H45" s="11" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="46" ht="46.95" customHeight="1" spans="1:19">
@@ -4131,7 +4149,7 @@
         <v>44</v>
       </c>
       <c r="B46" s="15" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C46" s="15" t="s">
         <v>9</v>
@@ -4141,16 +4159,16 @@
       </c>
       <c r="E46" s="16"/>
       <c r="F46" s="17" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="G46" s="17" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="H46" s="22" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="I46" s="1" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="47" ht="46.95" customHeight="1" spans="1:19">
@@ -4158,7 +4176,7 @@
         <v>45</v>
       </c>
       <c r="B47" s="15" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C47" s="15" t="s">
         <v>9</v>
@@ -4168,16 +4186,16 @@
       </c>
       <c r="E47" s="16"/>
       <c r="F47" s="15" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="G47" s="15" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="H47" s="22" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="I47" s="1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="48" ht="46.95" customHeight="1" spans="1:19">
@@ -4185,7 +4203,7 @@
         <v>46</v>
       </c>
       <c r="B48" s="15" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C48" s="15" t="s">
         <v>9</v>
@@ -4195,19 +4213,19 @@
       </c>
       <c r="E48" s="16"/>
       <c r="F48" s="17" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="G48" s="15" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="I48" s="1" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="S48" s="1" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="49" ht="46.95" customHeight="1" spans="1:19">
@@ -4215,7 +4233,7 @@
         <v>47</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C49" s="5" t="s">
         <v>9</v>
@@ -4225,13 +4243,13 @@
       </c>
       <c r="E49" s="6"/>
       <c r="F49" s="5" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="G49" s="5" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="H49" s="11" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
     </row>
     <row r="50" ht="46.95" customHeight="1" spans="1:19">
@@ -4239,7 +4257,7 @@
         <v>48</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C50" s="8" t="s">
         <v>26</v>
@@ -4249,7 +4267,7 @@
       <c r="F50" s="6"/>
       <c r="G50" s="6"/>
       <c r="H50" s="11" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="51" ht="46.95" customHeight="1" spans="1:19">
@@ -4257,7 +4275,7 @@
         <v>49</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C51" s="8" t="s">
         <v>26</v>
@@ -4275,7 +4293,7 @@
         <v>50</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C52" s="8" t="s">
         <v>9</v>
@@ -4285,19 +4303,19 @@
       </c>
       <c r="E52" s="6"/>
       <c r="F52" s="5" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="G52" s="5" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="I52" s="1" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="S52" s="1" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="53" ht="46.95" customHeight="1" spans="1:19">
@@ -4305,7 +4323,7 @@
         <v>51</v>
       </c>
       <c r="B53" s="8" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C53" s="8" t="s">
         <v>9</v>
@@ -4315,13 +4333,13 @@
       </c>
       <c r="E53" s="6"/>
       <c r="F53" s="23" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="G53" s="5" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="H53" s="24" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="54" ht="46.95" customHeight="1" spans="1:19">
@@ -4329,7 +4347,7 @@
         <v>52</v>
       </c>
       <c r="B54" s="8" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C54" s="8" t="s">
         <v>9</v>
@@ -4339,13 +4357,13 @@
       </c>
       <c r="E54" s="6"/>
       <c r="F54" s="5" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="G54" s="5" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="H54" s="22" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="55" ht="46.95" customHeight="1" spans="1:19">
@@ -4353,7 +4371,7 @@
         <v>53</v>
       </c>
       <c r="B55" s="8" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C55" s="8" t="s">
         <v>9</v>
@@ -4363,16 +4381,16 @@
       </c>
       <c r="E55" s="6"/>
       <c r="F55" s="5" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="G55" s="5" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="H55" s="18" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="K55" s="11" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="56" ht="46.95" customHeight="1" spans="1:19">
@@ -4380,7 +4398,7 @@
         <v>54</v>
       </c>
       <c r="B56" s="8" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C56" s="8" t="s">
         <v>9</v>
@@ -4390,16 +4408,16 @@
       </c>
       <c r="E56" s="6"/>
       <c r="F56" s="5" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="G56" s="5" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="H56" s="18" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="K56" s="11" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
     </row>
     <row r="57" ht="46.95" customHeight="1" spans="1:19">
@@ -4407,7 +4425,7 @@
         <v>55</v>
       </c>
       <c r="B57" s="8" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C57" s="8" t="s">
         <v>9</v>
@@ -4417,13 +4435,13 @@
       </c>
       <c r="E57" s="6"/>
       <c r="F57" s="5" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="G57" s="5" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="58" ht="46.95" customHeight="1" spans="1:19">
@@ -4431,7 +4449,7 @@
         <v>56</v>
       </c>
       <c r="B58" s="8" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C58" s="8" t="s">
         <v>9</v>
@@ -4441,13 +4459,13 @@
       </c>
       <c r="E58" s="6"/>
       <c r="F58" s="5" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="G58" s="5" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="59" ht="46.95" customHeight="1" spans="1:19">
@@ -4455,7 +4473,7 @@
         <v>57</v>
       </c>
       <c r="B59" s="17" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C59" s="17" t="s">
         <v>9</v>
@@ -4465,13 +4483,13 @@
       </c>
       <c r="E59" s="16"/>
       <c r="F59" s="17" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="G59" s="15" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="H59" s="22" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="60" ht="46.95" customHeight="1" spans="1:19">
@@ -4479,7 +4497,7 @@
         <v>58</v>
       </c>
       <c r="B60" s="17" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C60" s="17" t="s">
         <v>9</v>
@@ -4489,13 +4507,13 @@
       </c>
       <c r="E60" s="16"/>
       <c r="F60" s="17" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="G60" s="17" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="H60" s="22" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="61" ht="46.95" customHeight="1" spans="1:19">
@@ -4503,7 +4521,7 @@
         <v>59</v>
       </c>
       <c r="B61" s="15" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C61" s="15" t="s">
         <v>9</v>
@@ -4513,16 +4531,16 @@
       </c>
       <c r="E61" s="16"/>
       <c r="F61" s="17" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="G61" s="17" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="K61" s="11" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="P61" s="1" t="s">
         <v>43</v>
@@ -4533,7 +4551,7 @@
         <v>60</v>
       </c>
       <c r="B62" s="17" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C62" s="17" t="s">
         <v>9</v>
@@ -4543,16 +4561,16 @@
       </c>
       <c r="E62" s="16"/>
       <c r="F62" s="17" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="G62" s="15" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="H62" s="18" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="K62" s="11" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="P62" s="1" t="s">
         <v>40</v>
@@ -4563,7 +4581,7 @@
         <v>61</v>
       </c>
       <c r="B63" s="15" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C63" s="15" t="s">
         <v>9</v>
@@ -4573,16 +4591,16 @@
       </c>
       <c r="E63" s="16"/>
       <c r="F63" s="17" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="G63" s="17" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="H63" s="18" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="P63" s="1" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
     <row r="64" ht="46.95" customHeight="1" spans="1:19">
@@ -4590,7 +4608,7 @@
         <v>62</v>
       </c>
       <c r="B64" s="17" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C64" s="17" t="s">
         <v>9</v>
@@ -4600,16 +4618,16 @@
       </c>
       <c r="E64" s="16"/>
       <c r="F64" s="17" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="G64" s="15" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="H64" s="18" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="P64" s="1" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="65" ht="46.95" customHeight="1" spans="1:20">
@@ -4617,7 +4635,7 @@
         <v>63</v>
       </c>
       <c r="B65" s="15" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C65" s="15" t="s">
         <v>26</v>
@@ -4627,7 +4645,7 @@
       <c r="F65" s="16"/>
       <c r="G65" s="16"/>
       <c r="H65" s="11" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="66" ht="46.95" customHeight="1" spans="1:20">
@@ -4635,7 +4653,7 @@
         <v>64</v>
       </c>
       <c r="B66" s="15" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C66" s="15" t="s">
         <v>26</v>
@@ -4653,24 +4671,24 @@
         <v>65</v>
       </c>
       <c r="B67" s="17" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C67" s="17" t="s">
         <v>9</v>
       </c>
       <c r="D67" s="17" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="E67" s="16"/>
       <c r="F67" s="17" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="G67" s="16"/>
       <c r="H67" s="1" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="K67" s="11" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="S67" s="18" t="s">
         <v>40</v>
@@ -4681,24 +4699,24 @@
         <v>66</v>
       </c>
       <c r="B68" s="17" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="C68" s="17" t="s">
         <v>9</v>
       </c>
       <c r="D68" s="17" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="E68" s="16"/>
       <c r="F68" s="17" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="G68" s="16"/>
       <c r="H68" s="1" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="K68" s="11" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="S68" s="18" t="s">
         <v>43</v>
@@ -4709,21 +4727,21 @@
         <v>67</v>
       </c>
       <c r="B69" s="8" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C69" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D69" s="8" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="E69" s="6"/>
       <c r="F69" s="25" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="G69" s="6"/>
       <c r="H69" s="18" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="70" ht="46.95" customHeight="1" spans="1:20">
@@ -4731,21 +4749,21 @@
         <v>68</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C70" s="5" t="s">
         <v>9</v>
       </c>
       <c r="D70" s="5" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="E70" s="6"/>
       <c r="F70" s="5" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="G70" s="6"/>
       <c r="H70" s="18" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="71" ht="46.95" customHeight="1" spans="1:20">
@@ -4753,7 +4771,7 @@
         <v>69</v>
       </c>
       <c r="B71" s="8" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C71" s="8" t="s">
         <v>9</v>
@@ -4763,19 +4781,19 @@
       </c>
       <c r="E71" s="6"/>
       <c r="F71" s="5" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="G71" s="8" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="H71" s="1" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="I71" s="1" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="S71" s="22" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
     </row>
     <row r="72" ht="46.95" customHeight="1" spans="1:20">
@@ -4783,29 +4801,29 @@
         <v>70</v>
       </c>
       <c r="B72" s="8" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="C72" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D72" s="8" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="E72" s="6"/>
       <c r="F72" s="5" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="G72" s="5" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="H72" s="1" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="I72" s="1" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="S72" s="22" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="73" ht="46.95" customHeight="1" spans="1:20">
@@ -4813,23 +4831,23 @@
         <v>71</v>
       </c>
       <c r="B73" s="8" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C73" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D73" s="8" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="E73" s="6"/>
       <c r="F73" s="5" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="G73" s="5" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="S73" s="22" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="74" ht="46.95" customHeight="1" spans="1:20">
@@ -4837,26 +4855,26 @@
         <v>72</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C74" s="5" t="s">
         <v>9</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E74" s="6"/>
       <c r="F74" s="5" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="G74" s="5" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="H74" s="1" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="S74" s="22" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="75" ht="46.95" customHeight="1" spans="1:20">
@@ -4864,26 +4882,26 @@
         <v>73</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C75" s="5" t="s">
         <v>9</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E75" s="6"/>
       <c r="F75" s="5" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="G75" s="5" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="H75" s="1" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="S75" s="22" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="76" ht="46.95" customHeight="1" spans="1:20">
@@ -4891,7 +4909,7 @@
         <v>74</v>
       </c>
       <c r="B76" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C76" s="8" t="s">
         <v>26</v>
@@ -4901,7 +4919,7 @@
       <c r="F76" s="6"/>
       <c r="G76" s="6"/>
       <c r="H76" s="11" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="77" ht="46.95" customHeight="1" spans="1:20">
@@ -4909,7 +4927,7 @@
         <v>75</v>
       </c>
       <c r="B77" s="8" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C77" s="8" t="s">
         <v>26</v>
@@ -4927,23 +4945,23 @@
         <v>76</v>
       </c>
       <c r="B78" s="8" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C78" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D78" s="8" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="E78" s="8" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="F78" s="5" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="G78" s="6"/>
       <c r="H78" s="11" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="79" ht="46.95" customHeight="1" spans="1:20">
@@ -4951,23 +4969,23 @@
         <v>77</v>
       </c>
       <c r="B79" s="8" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C79" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D79" s="8" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="E79" s="8" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="F79" s="8" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="G79" s="6"/>
       <c r="H79" s="11" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="80" ht="46.95" customHeight="1" spans="1:20">
@@ -4975,23 +4993,23 @@
         <v>78</v>
       </c>
       <c r="B80" s="8" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C80" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D80" s="8" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="E80" s="8" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="F80" s="26" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="G80" s="6"/>
       <c r="H80" s="24" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="T80" s="22"/>
     </row>
@@ -5000,7 +5018,7 @@
         <v>79</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C81" s="5" t="s">
         <v>9</v>
@@ -5010,7 +5028,7 @@
       </c>
       <c r="E81" s="6"/>
       <c r="F81" s="27" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="G81" s="6"/>
       <c r="H81" s="28"/>
@@ -5021,21 +5039,21 @@
         <v>80</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="C82" s="5" t="s">
         <v>9</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="E82" s="6"/>
       <c r="F82" s="27" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="G82" s="6"/>
       <c r="H82" s="28" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="T82" s="22"/>
     </row>
@@ -5044,7 +5062,7 @@
         <v>81</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C83" s="5" t="s">
         <v>9</v>
@@ -5054,11 +5072,11 @@
       </c>
       <c r="E83" s="6"/>
       <c r="F83" s="5" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="G83" s="6"/>
       <c r="H83" s="1" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="84" ht="46.95" customHeight="1" spans="1:20">
@@ -5066,7 +5084,7 @@
         <v>82</v>
       </c>
       <c r="B84" s="17" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C84" s="17" t="s">
         <v>9</v>
@@ -5076,11 +5094,11 @@
       </c>
       <c r="E84" s="16"/>
       <c r="F84" s="17" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="G84" s="16"/>
       <c r="H84" s="22" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
     </row>
     <row r="85" ht="46.95" customHeight="1" spans="1:20">
@@ -5088,7 +5106,7 @@
         <v>83</v>
       </c>
       <c r="B85" s="15" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="C85" s="15" t="s">
         <v>9</v>
@@ -5098,14 +5116,14 @@
       </c>
       <c r="E85" s="16"/>
       <c r="F85" s="17" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="G85" s="16"/>
       <c r="H85" s="18" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="K85" s="11" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="86" ht="46.95" customHeight="1" spans="1:20">
@@ -5113,7 +5131,7 @@
         <v>84</v>
       </c>
       <c r="B86" s="15" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="C86" s="15" t="s">
         <v>9</v>
@@ -5123,11 +5141,11 @@
       </c>
       <c r="E86" s="16"/>
       <c r="F86" s="17" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="G86" s="16"/>
       <c r="H86" s="1" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
     </row>
     <row r="87" ht="46.95" customHeight="1" spans="1:20">
@@ -5135,7 +5153,7 @@
         <v>85</v>
       </c>
       <c r="B87" s="15" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="C87" s="15" t="s">
         <v>9</v>
@@ -5145,11 +5163,11 @@
       </c>
       <c r="E87" s="16"/>
       <c r="F87" s="17" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="G87" s="16"/>
       <c r="H87" s="22" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
     </row>
     <row r="88" ht="46.95" customHeight="1" spans="1:20">
@@ -5157,7 +5175,7 @@
         <v>86</v>
       </c>
       <c r="B88" s="17" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="C88" s="17" t="s">
         <v>9</v>
@@ -5167,11 +5185,11 @@
       </c>
       <c r="E88" s="16"/>
       <c r="F88" s="17" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="G88" s="16"/>
       <c r="H88" s="22" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="89" ht="46.95" customHeight="1" spans="1:20">
@@ -5179,7 +5197,7 @@
         <v>87</v>
       </c>
       <c r="B89" s="15" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="C89" s="15" t="s">
         <v>9</v>
@@ -5189,7 +5207,7 @@
       </c>
       <c r="E89" s="16"/>
       <c r="F89" s="29" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="G89" s="16"/>
       <c r="H89" s="28"/>
@@ -5200,7 +5218,7 @@
         <v>88</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="C90" s="5" t="s">
         <v>9</v>
@@ -5210,11 +5228,11 @@
       </c>
       <c r="E90" s="6"/>
       <c r="F90" s="27" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="G90" s="6"/>
       <c r="H90" s="28" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="T90" s="22"/>
     </row>
@@ -5223,7 +5241,7 @@
         <v>89</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="C91" s="5" t="s">
         <v>9</v>
@@ -5233,11 +5251,11 @@
       </c>
       <c r="E91" s="6"/>
       <c r="F91" s="5" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="G91" s="6"/>
       <c r="H91" s="22" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
     </row>
     <row r="92" ht="46.95" customHeight="1" spans="1:20">
@@ -5245,7 +5263,7 @@
         <v>90</v>
       </c>
       <c r="B92" s="8" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C92" s="8" t="s">
         <v>9</v>
@@ -5254,14 +5272,14 @@
         <v>10</v>
       </c>
       <c r="E92" s="30" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="F92" s="5" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="G92" s="6"/>
       <c r="H92" s="22" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="93" ht="46.95" customHeight="1" spans="1:20">
@@ -5269,25 +5287,25 @@
         <v>91</v>
       </c>
       <c r="B93" s="8" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="C93" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D93" s="8" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="E93" s="31" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="F93" s="5" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="G93" s="5" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="H93" s="22" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
     </row>
     <row r="94" ht="46.95" customHeight="1" spans="1:20">
@@ -5295,21 +5313,21 @@
         <v>92</v>
       </c>
       <c r="B94" s="8" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C94" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D94" s="8" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="E94" s="6"/>
       <c r="F94" s="5" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="G94" s="6"/>
       <c r="H94" s="22" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
     </row>
     <row r="95" ht="46.95" customHeight="1" spans="1:20">
@@ -5317,25 +5335,25 @@
         <v>93</v>
       </c>
       <c r="B95" s="17" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="C95" s="17" t="s">
         <v>9</v>
       </c>
       <c r="D95" s="17" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="E95" s="17" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="F95" s="17" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="G95" s="17" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="H95" s="22" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="96" ht="46.95" customHeight="1" spans="1:20">
@@ -5343,21 +5361,21 @@
         <v>94</v>
       </c>
       <c r="B96" s="15" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="C96" s="15" t="s">
         <v>9</v>
       </c>
       <c r="D96" s="15" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="E96" s="16"/>
       <c r="F96" s="17" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="G96" s="16"/>
       <c r="H96" s="22" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
     </row>
     <row r="97" ht="46.95" customHeight="1" spans="1:9">
@@ -5365,23 +5383,23 @@
         <v>95</v>
       </c>
       <c r="B97" s="17" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="C97" s="17" t="s">
         <v>9</v>
       </c>
       <c r="D97" s="17" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="E97" s="17" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="F97" s="17" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="G97" s="16"/>
       <c r="H97" s="11" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="98" ht="46.95" customHeight="1" spans="1:9">
@@ -5389,21 +5407,21 @@
         <v>96</v>
       </c>
       <c r="B98" s="17" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="C98" s="17" t="s">
         <v>9</v>
       </c>
       <c r="D98" s="17" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="E98" s="16"/>
       <c r="F98" s="17" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="G98" s="16"/>
       <c r="H98" s="22" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="99" ht="46.95" customHeight="1" spans="1:9">
@@ -5411,7 +5429,7 @@
         <v>97</v>
       </c>
       <c r="B99" s="15" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C99" s="15" t="s">
         <v>9</v>
@@ -5421,14 +5439,14 @@
       </c>
       <c r="E99" s="16"/>
       <c r="F99" s="17" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="G99" s="16"/>
       <c r="H99" s="22" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="I99" s="22" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
     </row>
     <row r="100" ht="46.95" customHeight="1" spans="1:9">
@@ -5436,7 +5454,7 @@
         <v>98</v>
       </c>
       <c r="B100" s="5" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="C100" s="5" t="s">
         <v>9</v>
@@ -5446,14 +5464,14 @@
       </c>
       <c r="E100" s="6"/>
       <c r="F100" s="5" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="G100" s="6"/>
       <c r="H100" s="22" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="I100" s="22" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="101" ht="46.95" customHeight="1" spans="1:9">
@@ -5461,7 +5479,7 @@
         <v>99</v>
       </c>
       <c r="B101" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C101" s="5" t="s">
         <v>26</v>
@@ -5471,7 +5489,7 @@
       <c r="F101" s="6"/>
       <c r="G101" s="6"/>
       <c r="H101" s="11" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="102" ht="46.95" customHeight="1" spans="1:9">
@@ -5479,7 +5497,7 @@
         <v>100</v>
       </c>
       <c r="B102" s="5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C102" s="5" t="s">
         <v>26</v>

</xml_diff>

<commit_message>
STM32 power rail switch
</commit_message>
<xml_diff>
--- a/kicad/main/STM32G473VCT6_IOs.xlsx
+++ b/kicad/main/STM32G473VCT6_IOs.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11580" tabRatio="500"/>
+    <workbookView windowWidth="28800" windowHeight="12180" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Table 1" sheetId="1" r:id="rId1"/>
@@ -1261,6 +1261,9 @@
     <t>TIM8_CH1N, UART4_TX, SPI3_SCK/I2S3_CK, USART3_TX, EVENTOUT</t>
   </si>
   <si>
+    <t>USB_PWR_EN</t>
+  </si>
+  <si>
     <t>PC11</t>
   </si>
   <si>
@@ -1377,7 +1380,7 @@
     <t>JTDO-TRACESWO, TIM2_CH2, TIM4_ETR, UCPD1_CRS_SYNC, TIM8_CH1N, SPI1_SCK, SPI3_SCK/I2S3_CK, USART2_TX, TIM3_ETR, FDCAN3_RX, SAI1_SCK_B, EVENTOUT</t>
   </si>
   <si>
-    <t>IMU-SPI-SCLK</t>
+    <t>3.3V_EN</t>
   </si>
   <si>
     <t>PB4</t>
@@ -1476,7 +1479,7 @@
     <t>UCPD1_CC2</t>
   </si>
   <si>
-    <t>IMU-SPI-MISO</t>
+    <t>5V_EN</t>
   </si>
   <si>
     <t>PB5</t>
@@ -1485,7 +1488,7 @@
     <t>TIM16_BKIN, TIM3_CH2, TIM8_CH3N, I2C1_SMBA, SPI1_MOSI, SPI3_MOSI/I2S3_SD, USART2_CK, I2C3_SDA, FDCAN2_RX, TIM17_CH1 , LPTIM1_IN1 , SAI1_SD_B, UART5_CTS, EVENTOUT</t>
   </si>
   <si>
-    <t>IMU-SPI-MOSI</t>
+    <t>PI_DONE</t>
   </si>
   <si>
     <t>PB6</t>
@@ -1522,9 +1525,6 @@
   </si>
   <si>
     <t>UCPD1_CC1</t>
-  </si>
-  <si>
-    <t>IMU-SPI-CS</t>
   </si>
   <si>
     <t>PB7</t>
@@ -1855,12 +1855,18 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="6"/>
+      <name val="Arial MT"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <vertAlign val="superscript"/>
       <sz val="8"/>
       <name val="Arial MT"/>
       <charset val="1"/>
     </font>
     <font>
+      <vertAlign val="superscript"/>
       <sz val="6"/>
       <name val="Arial MT"/>
       <charset val="1"/>
@@ -1868,12 +1874,6 @@
     <font>
       <sz val="8"/>
       <color rgb="FF282828"/>
-      <name val="Arial MT"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <vertAlign val="superscript"/>
-      <sz val="6"/>
       <name val="Arial MT"/>
       <charset val="1"/>
     </font>
@@ -5034,7 +5034,9 @@
         <v>290</v>
       </c>
       <c r="G81" s="6"/>
-      <c r="H81" s="28"/>
+      <c r="H81" s="28" t="s">
+        <v>291</v>
+      </c>
       <c r="T81" s="22"/>
     </row>
     <row r="82" ht="46.95" customHeight="1" spans="1:20">
@@ -5042,7 +5044,7 @@
         <v>80</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C82" s="5" t="s">
         <v>9</v>
@@ -5052,11 +5054,11 @@
       </c>
       <c r="E82" s="6"/>
       <c r="F82" s="27" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="G82" s="6"/>
       <c r="H82" s="28" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="T82" s="22"/>
     </row>
@@ -5065,7 +5067,7 @@
         <v>81</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C83" s="5" t="s">
         <v>9</v>
@@ -5075,11 +5077,11 @@
       </c>
       <c r="E83" s="6"/>
       <c r="F83" s="5" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="G83" s="6"/>
       <c r="H83" s="1" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="84" ht="46.95" customHeight="1" spans="1:20">
@@ -5087,7 +5089,7 @@
         <v>82</v>
       </c>
       <c r="B84" s="17" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C84" s="17" t="s">
         <v>9</v>
@@ -5097,11 +5099,11 @@
       </c>
       <c r="E84" s="16"/>
       <c r="F84" s="17" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="G84" s="16"/>
       <c r="H84" s="22" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="85" ht="46.95" customHeight="1" spans="1:20">
@@ -5109,7 +5111,7 @@
         <v>83</v>
       </c>
       <c r="B85" s="15" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C85" s="15" t="s">
         <v>9</v>
@@ -5119,14 +5121,14 @@
       </c>
       <c r="E85" s="16"/>
       <c r="F85" s="17" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="G85" s="16"/>
       <c r="H85" s="18" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="K85" s="11" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="86" ht="46.95" customHeight="1" spans="1:20">
@@ -5134,7 +5136,7 @@
         <v>84</v>
       </c>
       <c r="B86" s="15" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C86" s="15" t="s">
         <v>9</v>
@@ -5144,11 +5146,11 @@
       </c>
       <c r="E86" s="16"/>
       <c r="F86" s="17" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="G86" s="16"/>
       <c r="H86" s="1" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="87" ht="46.95" customHeight="1" spans="1:20">
@@ -5156,7 +5158,7 @@
         <v>85</v>
       </c>
       <c r="B87" s="15" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C87" s="15" t="s">
         <v>9</v>
@@ -5166,11 +5168,11 @@
       </c>
       <c r="E87" s="16"/>
       <c r="F87" s="17" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="G87" s="16"/>
       <c r="H87" s="22" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="88" ht="46.95" customHeight="1" spans="1:20">
@@ -5178,7 +5180,7 @@
         <v>86</v>
       </c>
       <c r="B88" s="17" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C88" s="17" t="s">
         <v>9</v>
@@ -5188,11 +5190,11 @@
       </c>
       <c r="E88" s="16"/>
       <c r="F88" s="17" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="G88" s="16"/>
       <c r="H88" s="22" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="89" ht="46.95" customHeight="1" spans="1:20">
@@ -5200,7 +5202,7 @@
         <v>87</v>
       </c>
       <c r="B89" s="15" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C89" s="15" t="s">
         <v>9</v>
@@ -5210,11 +5212,11 @@
       </c>
       <c r="E89" s="16"/>
       <c r="F89" s="29" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="G89" s="16"/>
       <c r="H89" s="24" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="T89" s="22"/>
     </row>
@@ -5223,7 +5225,7 @@
         <v>88</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C90" s="5" t="s">
         <v>9</v>
@@ -5233,11 +5235,11 @@
       </c>
       <c r="E90" s="6"/>
       <c r="F90" s="27" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="G90" s="6"/>
       <c r="H90" s="28" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="T90" s="22"/>
     </row>
@@ -5246,7 +5248,7 @@
         <v>89</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C91" s="5" t="s">
         <v>9</v>
@@ -5256,11 +5258,11 @@
       </c>
       <c r="E91" s="6"/>
       <c r="F91" s="5" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="G91" s="6"/>
       <c r="H91" s="22" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="92" ht="46.95" customHeight="1" spans="1:20">
@@ -5268,7 +5270,7 @@
         <v>90</v>
       </c>
       <c r="B92" s="8" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C92" s="8" t="s">
         <v>9</v>
@@ -5277,14 +5279,14 @@
         <v>10</v>
       </c>
       <c r="E92" s="30" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F92" s="5" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="G92" s="6"/>
       <c r="H92" s="22" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="93" ht="46.95" customHeight="1" spans="1:20">
@@ -5292,25 +5294,25 @@
         <v>91</v>
       </c>
       <c r="B93" s="8" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C93" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D93" s="8" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E93" s="31" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F93" s="5" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="G93" s="5" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="H93" s="22" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="94" ht="46.95" customHeight="1" spans="1:20">
@@ -5318,7 +5320,7 @@
         <v>92</v>
       </c>
       <c r="B94" s="8" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C94" s="8" t="s">
         <v>9</v>
@@ -5328,11 +5330,11 @@
       </c>
       <c r="E94" s="6"/>
       <c r="F94" s="5" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="G94" s="6"/>
       <c r="H94" s="22" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="95" ht="46.95" customHeight="1" spans="1:20">
@@ -5340,26 +5342,24 @@
         <v>93</v>
       </c>
       <c r="B95" s="17" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C95" s="17" t="s">
         <v>9</v>
       </c>
       <c r="D95" s="17" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E95" s="17" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="F95" s="17" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="G95" s="17" t="s">
-        <v>337</v>
-      </c>
-      <c r="H95" s="22" t="s">
         <v>338</v>
       </c>
+      <c r="H95" s="22"/>
     </row>
     <row r="96" ht="46.95" customHeight="1" spans="1:20">
       <c r="A96" s="14">

</xml_diff>